<commit_message>
Changes made to bell ring mode. Added Questions for bell ring.
</commit_message>
<xml_diff>
--- a/question/question.xlsx
+++ b/question/question.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\Maths-Tutor-QT-V2\question\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDHANT\Desktop\Zendalona\forkedFolder\Maths-Tutor-QT-V2\question\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{360D72E5-C25E-48AC-9517-042DA4287FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF4E48A-16B9-43FA-A443-77345EDBC0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="78">
   <si>
     <t>question</t>
   </si>
@@ -234,23 +234,38 @@
     <t>Remainder</t>
   </si>
   <si>
-    <t>Ramu has {x} apples</t>
-  </si>
-  <si>
     <t>Bellring</t>
   </si>
   <si>
-    <t>x1:5</t>
-  </si>
-  <si>
-    <t>{x}</t>
+    <t xml:space="preserve">{a} + {b} = </t>
+  </si>
+  <si>
+    <t>{a} + {b} =</t>
+  </si>
+  <si>
+    <t>a1:9*b1:9*</t>
+  </si>
+  <si>
+    <t>a2:5*b2:5*</t>
+  </si>
+  <si>
+    <t>a2;1;4*b1:5*</t>
+  </si>
+  <si>
+    <t>a3;1;3*b1:3*</t>
+  </si>
+  <si>
+    <t>a2;1;4*b2;1;1*</t>
+  </si>
+  <si>
+    <t>a5;1;1*b1:9*</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -259,11 +274,21 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -286,10 +311,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -606,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="107.21875" customWidth="1"/>
@@ -616,542 +643,662 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>2</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="A4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>2</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="2">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="2">
         <v>3</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="2">
         <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="D15" s="2">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>2</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="D17" s="2">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>2</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="2">
         <v>3</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="D20" s="2">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="2">
         <v>2</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="2">
         <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="2">
         <v>2</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="2">
         <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="2">
         <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="2">
         <v>2</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="A26" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="E26" t="s">
+      <c r="D26" s="2">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="A27" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D27" s="2">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="2">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="2">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F29" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="2">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C27" t="s">
+      <c r="B31" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="2">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F32" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
-      <c r="E27" t="s">
-        <v>72</v>
-      </c>
-      <c r="F27">
+      <c r="B33" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D33" s="2">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" s="2">
         <v>10</v>
       </c>
     </row>

</xml_diff>